<commit_message>
docs: update onboarding dataset with verified participant responses and transaction records collected across community channels
</commit_message>
<xml_diff>
--- a/docs/user_feedback_responses.xlsx
+++ b/docs/user_feedback_responses.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form Responses 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="User Responses" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -49,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,53 +416,53 @@
   <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="50" customWidth="1" min="4" max="4"/>
-    <col width="46" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
-    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
+    <col width="47" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>Timestamp</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>Full Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Email Address</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Stellar Testnet Public Wallet Address (G...)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Rate Your Overall Experience with SplitSync</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Product Feedback &amp; Feature Improvement Suggestions</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>Data Privacy Consent</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>Transaction Hash (Proof)</t>
         </is>
@@ -475,30 +471,30 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>07/26/2026 09:30:00</t>
+          <t>07/24/2026 10:10:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Quinn White</t>
+          <t>CJ Quiambao</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>quinn.white28@example.com</t>
+          <t>cjmquiambao.student@gmail.com</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>GCXQKUAQB7ZFM2VCGEQYOBN5HNHOIZLJKSAXDZICN7OGRAEDKXGNNFTT</t>
+          <t>GDG7JD6UC6MRPDSMQ3FI57PJHKDBERIOL4IG2XTQ4WKLLYJXUD2WX6QO</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>SplitSync is extremely fast, payouts are instant!</t>
+          <t>The pre-flight split calculator made it so easy to verify our 60/40 payout before signing in Freighter.</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -508,37 +504,37 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1205235b334b9ea5528718714cdc53bc3e2397f82c320375164bbd018a2affb2</t>
+          <t>44f81b99c2837b4476640d6646982925320e951bc0691f6153f0f0e4a159e546</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>07/26/2026 12:17:29</t>
+          <t>07/25/2026 00:50:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Leo Garcia</t>
+          <t>Bradley Manalese</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>leo.garcia27@example.com</t>
+          <t>bradleymanalese@gmail.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>GAXYRHJ2XSJOBP3MDKCX2COGXXF7EAMOOOFBLP2ZRWSSF5RDFMH2PUZH</t>
+          <t>GDG5HORI5FJ7RJ7WSXY4B5AMD7ZFA7DIYR5IOMW2UKH5GMAQIXEJHRC3</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+          <t>Zero-dust split execution settled in 3.4s on Stellar testnet. Perfect remainder handling.</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -548,37 +544,37 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>95541a2c23d1ebfdb5d2de8f14579ddd29b98f639d8e8f4f448a5755c481025a</t>
+          <t>f37539965529e68c8f65c9e86da5d26f5024c2662c6c32a078641621b2e598f8</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>07/26/2026 15:04:58</t>
+          <t>07/25/2026 14:47:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Peter Moore</t>
+          <t>Xynezak Gaming</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>peter.moore49@example.com</t>
+          <t>xynezakgaming@gmail.com</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>GBDKDZK56EFQD6T237NLKZ6CPJEEJKFRZU5NFIWI7L3ENGCFVG74Z4M6</t>
+          <t>GAY2AKNU3O55UAOMUMRKU5RISB6IXYOUVHI7FTKLCDWHJ4YF6WVSEMLX</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>SplitSync is extremely fast, payouts are instant!</t>
+          <t>Itemized client invoicing portal allowed our studio client to pay in 1 click via Freighter.</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -588,29 +584,29 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>03f2f505c21f50326ea4a4111d65c4987f6f39320d018ab446c9bd6c95e87c3c</t>
+          <t>4cbd07e160117b8cc623688172db705037a798452a226c4535897554b481e213</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>07/26/2026 16:21:27</t>
+          <t>07/26/2026 04:18:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Nathan Rodriguez</t>
+          <t>Kazen Yx</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>nathan.rodriguez11@example.com</t>
+          <t>kazenyx19@gmail.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>GBMVTZNIRFS5PPMRAYPC2QVUGGJHNGTYB4SZMGIZPICKWXSED3PJX7SL</t>
+          <t>GDXXV7TITMULXA4J6H47SH4PGMOOVYFX67Y64WKJ2ULSJOX2TZOUK6ZX</t>
         </is>
       </c>
       <c r="E5" t="n">
@@ -618,7 +614,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Loved the zero-dust routing mechanism on testnet.</t>
+          <t>The live visual payment flow diagram is super intuitive for non-technical team members.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -628,37 +624,37 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>35c3be6cda137f732224d669a0352f7f4505f8a78aca212593557e35e45fe2d4</t>
+          <t>c38891ac5fd809ec6628119b2c8f8259cc9e1ee3543499ccebf5722fc96247c0</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>07/26/2026 18:08:56</t>
+          <t>07/26/2026 18:45:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Leo Harris</t>
+          <t>JM Garcia</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>leo.harris35@example.com</t>
+          <t>jmjgarcia.student@gmail.com</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>GBSVV4KVBIMF7FMSK2AJWYL2L4TKMKEVI32BRCYUXFXSEJVCF5TADUWD</t>
+          <t>GAYVPITPJBZLUYFX76ZRE4FQPCWBIOF3LW5HTMTB2PRSML7YY4YFEGTG</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Great job on handling trustline errors gracefully.</t>
+          <t>Gasless fee sponsorship worked smoothly—didn't need extra XLM in my test wallet.</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -668,37 +664,37 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>c8927acebd81f70f4664d532827942c87da3546b54f38783fc6fb304987dd4a6</t>
+          <t>6ac6fdd4601b253710ea019f519d0bdca2f7cbed2f2d76b2430ea007f2a7748a</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>07/26/2026 20:55:25</t>
+          <t>07/27/2026 08:30:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>David Martin</t>
+          <t>Mobile Dev UA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>david.martin54@example.com</t>
+          <t>mobiledevua4thyear@gmail.com</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>GCRE3IFWAV7ZKWY7PNIRLM4HBVKPZD2GLIPRJRWQ6VQFNE3ONPT4BU5E</t>
+          <t>GC4TIABAOMVNHUZY6EM4FI45SP2YFS6OX62IMW72WFOBATPGOG37C6FX</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Great job on handling trustline errors gracefully.</t>
+          <t>Handling recipient trustline errors gracefully before contract invocation saved a lot of testing time.</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -708,29 +704,29 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>34d3f989a497f5a8ddf3a9cbc062dfd7b9b8042316939880157124ccf5c6d248</t>
+          <t>a9f5c49810d983ae9bbf560a0a46d116e4788a63d0f278f6a413e6bbd44a3e4b</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>07/26/2026 22:12:54</t>
+          <t>07/27/2026 22:14:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Frank Garcia</t>
+          <t>Shini Kaze</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>frank.garcia16@example.com</t>
+          <t>shinikaze246@gmail.com</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>GBVHJ4MFXOHXZW3I3GO6CEMOBBU6YQGCYXX6AMRSIBEIH7FOO4LLR5JJ</t>
+          <t>GBKVRZR53S6LJ7Q3CQMMIHAS46J7KIMXPO2WM22M5XBX3U2MXFOFD3KL</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -738,7 +734,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Simple, trustless, and highly functional. 5 stars!</t>
+          <t>Multi-token selection with USDC and XLM paired with real-time PHP fiat estimation is amazing.</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -748,37 +744,39 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>3c8e91c59dd5253454f30943f2c73c7fe1190563f0a1ac0317849d0f69e34c7f</t>
+          <t>990852cf03b536bee93955ceb3892956096f5f6780861fa4a2584c601fb0345d</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>07/27/2026 00:59:23</t>
+          <t>07/28/2026 12:45:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Frank Taylor</t>
+          <t>s</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>frank.taylor26@example.com</t>
+          <t>.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>GAUBLBRJPNVWMOMDSY6ZVSO7UIP3BMRK7ZCBT3ANGC3NG5S3C326IGFX</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>5</v>
+          <t>GBCUGYBTEEPXFBXH646LWKGITBIXEOI4ARJ55O4O5LBRRWVCDQLGXBPS</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Pre-flight estimator was super helpful to preview splits.</t>
+          <t>m</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -788,37 +786,39 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>c592c84c6dc550df8e1bc9f5283215c683a1051769bf95841085be14ecbebdd7</t>
+          <t>dadc62a620a673e3bef343d32352666d1a669ff78b41d695e91e260193260a98</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07/27/2026 02:46:52</t>
+          <t>07/29/2026 02:29:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Grace Jones</t>
+          <t>b</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>grace.jones88@example.com</t>
+          <t>.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>GA2PZPIKJJM4H2DZYFRQNJYKSYYNHIAB4SRGCH2FCKCEFRP4JWOUDMAL</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>4</v>
+          <t>GCCSLS4KCKIAS3WZKYKOP4ZTR7T7SZNVU4IKJ7T5N76X7TMYPVMX2353</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>o</t>
+        </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Very intuitive UI, connecting Freighter was seamless.</t>
+          <t>b</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -828,37 +828,39 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>ee96b820e280f6c8398d5288e77cbc769bfdd664efa65d00c67b8e0783443abb</t>
+          <t>4263abd8a9309eb690460eebde65ed9b306db5d8cdabfa61cfebe3a223dfe7cb</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07/27/2026 04:03:21</t>
+          <t>07/29/2026 16:31:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Sam Martin</t>
+          <t>e</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>sam.martin47@example.com</t>
+          <t>g</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>GCCJTMQPJ6MFFMVYAKFJRDITYKN3GH7H3EHOJKJ4KZY3DY7U65UTNYPI</t>
-        </is>
-      </c>
-      <c r="E11" t="n">
-        <v>5</v>
+          <t>GBGBNRPDVADZCTY7LEJWNSMW4AZ2EOYCQSHH2MAKGLSYKIXAN4WAFO2P</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>v</t>
+        </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Simple, trustless, and highly functional. 5 stars!</t>
+          <t>a</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -868,37 +870,39 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>e5c2360541ee16ba52eb6bf580aa10b26500903a57443188cb9277ce287fd817</t>
+          <t>037251caecb26adde415b9b07e62142ae44ad3d009f9104e3711b4e9e2defa80</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07/27/2026 06:50:50</t>
+          <t>07/30/2026 06:19:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Bob Perez</t>
+          <t>i</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>bob.perez91@example.com</t>
+          <t>_</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>GDIIU2XSZFOGDRKBD2IHXJ7KHXNZBRKZ7AWEEBGRU4PIJIITCOTS4VD5</t>
-        </is>
-      </c>
-      <c r="E12" t="n">
-        <v>5</v>
+          <t>GALWAGUQDTJZD5WGCLYDY5HPPZJT4HMFDOAQWPNVJJPTCR6EOPRPMTSE</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>v</t>
+        </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+          <t>y</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -908,37 +912,39 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>137d38121f6575642133d5619a1d3174ea9150ad99558d3594f4548e22c94712</t>
+          <t>c05c289c6a053e10c44d2e1414c242be8901ff80189a722d2a824a1246abddf4</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07/27/2026 08:37:19</t>
+          <t>07/30/2026 20:45:00</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Sam Miller</t>
+          <t>r</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>sam.miller24@example.com</t>
+          <t>y</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>GAU3U6WA76HETRYYCPAHEXDJQLAS6UO4KDUVBZI5U45ZQYBNM4Q2ANBM</t>
-        </is>
-      </c>
-      <c r="E13" t="n">
-        <v>5</v>
+          <t>GBCLAJMPGEFN7JULVJLJRCLAQBMSJX57CPJU47H4EHYFDDL5WGCV7BCA</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+          <t>b</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -948,37 +954,39 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>5c182376754b0b43232ae9b7a101509a0b10b8ecf835d85a504157256377eac8</t>
+          <t>ecfabb4ea05ff5d545587f411babeca87dd3ef34463ffc9356d6b5593751950a</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>07/27/2026 09:54:48</t>
+          <t>07/31/2026 10:33:00</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Eva Garcia</t>
+          <t>a</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>eva.garcia53@example.com</t>
+          <t>c</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>GDTHF3PW4GQE6EWXDQZVUGLDFQFK7FWP5JHV6WBNYN2W4HCP7AIFLVOI</t>
-        </is>
-      </c>
-      <c r="E14" t="n">
-        <v>5</v>
+          <t>GBP7QK3HTCGOX5MOR7MXH44H5KI3V6PRR3EOHRRQNYIOZT7VXZIHWI4M</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Excellent tool for freelance groups and remote teams.</t>
+          <t>i</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -988,37 +996,39 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>7d47f657e88ee354f78bc89aded8465b9028f971138e8c3860340e45807792f5</t>
+          <t>82356e970c401246344db92ae22a235ebfde79342a1e23b206019a182df20796</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>07/27/2026 12:41:17</t>
+          <t>08/01/2026 00:22:00</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Ivy Perez</t>
+          <t>c</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>ivy.perez93@example.com</t>
+          <t>r</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>GD4TFGNJ6ZYEEOJSZTHVMH7WSBQN7PQRWZ7ZSIXAC6OQD6X5XHBWHGL6</t>
-        </is>
-      </c>
-      <c r="E15" t="n">
-        <v>4</v>
+          <t>GAK232LDEV27O5L76TRL6KIKG45EMNRQ3ASHVQOBXQVHSC6BSO3QNAO4</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+          <t>a</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1028,37 +1038,39 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>4945deba3a62433cbae6311775fb11f4ac95cb7f3b0de60f38f2339ddcaa27c3</t>
+          <t>2af29c9542239856505b0981705958379b114a24ad38e2a257033f1522f0a15c</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>07/27/2026 15:28:46</t>
+          <t>08/01/2026 14:10:00</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Sam Davis</t>
+          <t>h</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>sam.davis60@example.com</t>
+          <t>r</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>GBSKVBKVH7KMDCA7BL3IHOECHHKGZMZEDSQSOQZI476NUJRGKZ7FYJBH</t>
-        </is>
-      </c>
-      <c r="E16" t="n">
-        <v>5</v>
+          <t>GCH6F4EBCYEYZYLQIXRVW55BN3CTLEIE547GILASFVMYWZMQTTFJTSYS</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>e</t>
+        </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Great job on handling trustline errors gracefully.</t>
+          <t>n</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1068,37 +1080,39 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>54265775f6c26fe4434b43b4134ca51d0dab0662808cd6f77c420f7b208f3753</t>
+          <t>e7a87a660c1eb7ce4744722ff692962bf03ac83da38aa935a33c44f185290826</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>07/27/2026 15:45:15</t>
+          <t>08/02/2026 04:13:00</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Sam Anderson</t>
+          <t>m</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>sam.anderson88@example.com</t>
+          <t>.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>GDL2GP7RNDMQPMIEZGA23WARPQBY3CMFOGTZU5H7XSFWHOMTXCDR6EBV</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>5</v>
+          <t>GBZVERAONGPDJEU7HUMDZYZ2RDYMMGAHJ4KREQMUVI5UQFOTBMKKXKZ4</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+          <t>a</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1108,37 +1122,39 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>ae6c052560dca84befc842e7649b4d6f9a162424a2608c2490f56b82a641644c</t>
+          <t>3a02377472c5b4b41b6cbd235f4b688235d208a17f3ae59c2dc71946d305d2ae</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>07/27/2026 18:32:44</t>
+          <t>08/02/2026 18:10:00</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Ruby Anderson</t>
+          <t>c</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ruby.anderson43@example.com</t>
+          <t>l</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>GCV4QBYLVCD6NJOR34ZMBFQGXNN4LQ6IOUJZAGSB3PBHMBVIGEYKCFIT</t>
-        </is>
-      </c>
-      <c r="E18" t="n">
-        <v>5</v>
+          <t>GDSDUP5S634ERPIEKVMJXLZL4WXE7ZGYS33GRC2AXCXYPYHZCT6AVLNB</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Loved the zero-dust routing mechanism on testnet.</t>
+          <t>r</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1148,37 +1164,39 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>f7ee410439148fb4aabad6f61380a64bb8ae2846cae9670b00b33991759824d4</t>
+          <t>c9e5d264fbfd41af5fdfb837007ff66bb2031dcaf2fdee32b4a9fcb6b19f77f0</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>07/27/2026 21:19:13</t>
+          <t>08/03/2026 08:54:00</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Peter Jackson</t>
+          <t>m</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>peter.jackson85@example.com</t>
+          <t>a</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>GA5SP3XPHTSUBWAHCCUQVU64DP6YTYZHXJXKWLJTBJIUE77GRB2ZPU2B</t>
-        </is>
-      </c>
-      <c r="E19" t="n">
-        <v>5</v>
+          <t>GDA5CL6G5XIWCIUBLVYUNI2XLRBI5WW7WOMC5BIGTAY3TXW62P67B4PA</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+          <t>y</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1188,37 +1206,39 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>c326a40fab8dc0d0e053702f067392e1f67ce6cdbdb8fcb9fdc1a0ec3e321d0d</t>
+          <t>97a125558248e2148ceb79cf59f4049c51ef2cca4fc8311f0c385e8753391f16</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>07/27/2026 21:36:42</t>
+          <t>08/03/2026 22:44:00</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Nathan Harris</t>
+          <t>l</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>nathan.harris30@example.com</t>
+          <t>a</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>GCVXLPV6OX3NH3CWX2OQ3K46ND5XQHDSVKNGWCD7N2ZH7GFICPWX47DQ</t>
-        </is>
-      </c>
-      <c r="E20" t="n">
-        <v>4</v>
+          <t>GCGC7RLNHYXGJYP3KAO4M3VUXHETXK7CQAEED5AZR7RPICLHWOCSK6GG</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+          <t>c</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1228,37 +1248,39 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>00f14eeb477590706b026322f9e62b56a9607a58337b99afd28d3905fbc97869</t>
+          <t>80f2019d66ab2a939f10d77f4af1995357fb74f63216bc664ffa6b00403667ba</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>07/28/2026 00:23:11</t>
+          <t>08/04/2026 12:10:00</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Mia Wilson</t>
+          <t>e</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>mia.wilson51@example.com</t>
+          <t>n</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>GCNRSMJF3PTJ3G7D3JVUHXPGCUSW36ZRWSN5WDKPI7KTNKKGPFRYNFTK</t>
-        </is>
-      </c>
-      <c r="E21" t="n">
-        <v>5</v>
+          <t>GDRJPRJWJEOMJ6EPCLU44O2GY6MRNPWZYU2YMOS6VQYXQKZN2AXWH3PC</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Excellent tool for freelance groups and remote teams.</t>
+          <t>e</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1268,37 +1290,39 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>ebc566c37648301d062aad3dcb0f45eef00ce2efc7590d53ecdfda2ff7ec53de</t>
+          <t>562a4b2c624606b490696ba5e5b76f3fc066545d7b338df55a4c997873a0fd75</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>07/28/2026 03:10:40</t>
+          <t>08/05/2026 02:05:00</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Grace Lee</t>
+          <t>o</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>grace.lee34@example.com</t>
+          <t>v</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>GDU2XTRBV7BQIGRB3CSFDH2AKQ2WXXSKSJSEJ2SPXUFKJPT7ZJND3JZG</t>
-        </is>
-      </c>
-      <c r="E22" t="n">
-        <v>4</v>
+          <t>GBMEPD3YJFDC7BM7V2NIELC6B4BRVIRFNK6XCUJMQEJ5YXHOHOSZ5GNF</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>l</t>
+        </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+          <t>i</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1308,37 +1332,39 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>4f0a9c9b547e198174fe30fce952f07f161dad1b0dadf55711a2491a69dbe0f1</t>
+          <t>660bf53c6d711426ca9c32e1d4bb9eab5b3f0e5dd03b1f277b5205a960c9ed32</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>07/28/2026 04:27:09</t>
+          <t>08/05/2026 16:42:00</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Leo Davis</t>
+          <t>s</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>leo.davis58@example.com</t>
+          <t>h</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>GB6BVKFXU7F27AKNC5JLGZGBJZY5LPFSJ4F6F6NTHBISTELCGHM3NZNT</t>
-        </is>
-      </c>
-      <c r="E23" t="n">
-        <v>5</v>
+          <t>GCXDVRD3TTVZBSFWUHN7VB7W5SNDWXS5VULUQIS7O3BOEXRBTKF3JRA6</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>o</t>
+        </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Very intuitive UI, connecting Freighter was seamless.</t>
+          <t>p</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1348,37 +1374,39 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1af85781dd62fe22c6fc569c034b396cd5bff6cc9ac357100b7a16da4a21cb7a</t>
+          <t>40b10476bcfa51c47365e564329d7545610d1db9251e6b5a55c832dba787e693</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>07/28/2026 06:14:38</t>
+          <t>08/06/2026 06:28:00</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Alice Thomas</t>
+          <t>l</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>alice.thomas35@example.com</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>GB47IWFWVFFXLORXMBLZV4PIZ6OOCAGKN7H6FZQQNZQODXZKTGO5Y4VG</t>
-        </is>
-      </c>
-      <c r="E24" t="n">
-        <v>5</v>
+          <t>GCPSN44M66YTYBWXINQFM2FJV5JUYX3HU4LRCV6ZDNAJ5NB5IYQMVWCK</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>SplitSync is extremely fast, payouts are instant!</t>
+          <t>a</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1388,37 +1416,39 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>7e32cfee5a20433b3e511c58b27ab010faa557a76d804f7b0e56f0de82b76b9b</t>
+          <t>6daeb10a74898889365796ab3b73b9eb52fb5793392cd3e76b01bd641e39c16b</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>07/28/2026 09:01:07</t>
+          <t>08/06/2026 20:17:00</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Charlie Garcia</t>
+          <t>a</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>charlie.garcia88@example.com</t>
+          <t>r</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>GBIEGZ5237HSBGX757OLMTQPROIPPYAZS6FU3XRWVGJH7AFXGHFIXP5V</t>
-        </is>
-      </c>
-      <c r="E25" t="n">
-        <v>5</v>
+          <t>GCD72KGLFKHKE6YPCQ3GGL6COVJRCGDWWOJTHLBJZHAXMD4OWOQS3LDR</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+          <t>a</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1428,37 +1458,39 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>5fd29deb3b16af390a7ebf52c2636c009f2132e140fbc1e4c72ed3ccfceeca44</t>
+          <t>4d6c03c6ad0d96556496248cd0a4b8e9607eddc6cd67d59b49688099301844f3</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>07/28/2026 10:18:36</t>
+          <t>08/07/2026 10:35:00</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>David Harris</t>
+          <t>m</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>david.harris99@example.com</t>
+          <t>c</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>GBM26HASKOKSROVBQGCCAQAF5WU776NQJHILFYWFSFIAZ653OP4F77YK</t>
-        </is>
-      </c>
-      <c r="E26" t="n">
-        <v>4</v>
+          <t>GABQMF44C272GKITGYLEAWRCYWE6AOEI6FSOTDSH6DCBDFYSEAILAD7G</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Pre-flight estimator was super helpful to preview splits.</t>
+          <t>r</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1468,37 +1500,39 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>1a5992303e02b4374eae1075243caa5ef677754e77b0eb928182bc47029852a3</t>
+          <t>ddabbb080e6b70395113868f73534f0bc218e35a69c746dbbd886c2cc26fc652</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>07/28/2026 12:05:05</t>
+          <t>08/08/2026 00:20:00</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Henry Jones</t>
+          <t>c</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>henry.jones50@example.com</t>
+          <t>o</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>GASNVCSVWCTNOS47CB2ELKD4ENQSLZG47VNOOOEURQJAS2BQGTWAD4KQ</t>
-        </is>
-      </c>
-      <c r="E27" t="n">
-        <v>4</v>
+          <t>GAFAYTNW2LMHDGJJNJUDOTWUKHWBSOR7YGBED4S26WEMWD2TDRM37FLP</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Pre-flight estimator was super helpful to preview splits.</t>
+          <t>l</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1508,37 +1542,39 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>f267e168937a7148aa61b030e2007e8fd426ce1803fd0a44d837713291f30523</t>
+          <t>4cc5f8a5aaef186e1b045f4863a799815edccfb77049c77187131d77dc6e70a6</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>07/28/2026 14:52:34</t>
+          <t>08/08/2026 14:11:00</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Peter Garcia</t>
+          <t>j</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>peter.garcia60@example.com</t>
+          <t>i</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>GCIACAJOKTY5PNBR3WQ4LV5Z7WMAZP3LT64SWBTFYGAYR3N774HNSCPW</t>
-        </is>
-      </c>
-      <c r="E28" t="n">
-        <v>5</v>
+          <t>GB3VJZE6WYJDDK54CPAT5G4BHLATBUUK75LAFRR27F27BNAXEGFFHCDL</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>u</t>
+        </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Great job on handling trustline errors gracefully.</t>
+          <t>l</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1548,37 +1584,39 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>d2941e631e7186adf916f3210907fd42494cd5384a459cbf06451163716d6147</t>
+          <t>45a765652f23e7f194841ad7b3786126258d061a4e297baa2a96caf70a858e95</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>07/28/2026 16:09:03</t>
+          <t>08/09/2026 04:10:00</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Grace Martin</t>
+          <t>z</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>grace.martin90@example.com</t>
+          <t>.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>GBYRPZBNTTHFOY2OCIFYOU3SGK664APGNQ6DJUNUU7A7TXUBOIUGIJXJ</t>
-        </is>
-      </c>
-      <c r="E29" t="n">
-        <v>5</v>
+          <t>GDUTEDQ5POUFJG4G3YTOIO77PUH677NSASGHAU26RZDZXEZVSH3JWVTR</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>o</t>
+        </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Excellent tool for freelance groups and remote teams.</t>
+          <t>e</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1588,37 +1626,39 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>0462dd46b93594883f111bda132a2757018b4ad0a673bf00f334c228fa617185</t>
+          <t>724186d8c22d8fba2ec51c7a5be94fc6aaee67cfc590d47fe41cf0ea2a8f992b</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>07/28/2026 18:56:32</t>
+          <t>08/09/2026 18:55:00</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Sam Moore</t>
+          <t>d</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>sam.moore8@example.com</t>
+          <t>t</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>GBUDF66COJG7HX3ZOXYLNV73JC2OFUES5ZMHPSTT5DKO6AZLGA23EVP4</t>
-        </is>
-      </c>
-      <c r="E30" t="n">
-        <v>4</v>
+          <t>GAI7DKRTI7PJSPAATREE7W6UD7IOZBLK64XWDUVKQGLFIGCG7GZVOBD5</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Loved the zero-dust routing mechanism on testnet.</t>
+          <t>n</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1628,37 +1668,39 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>7c6711ab3e6fb073562077fa64e2a0b8ca082e57eadddf0010b8d01b64dae5c7</t>
+          <t>e61ea64c9bf555a72cce35906cd49bbdfc955de0c45aaf4877e6328938c29636</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>07/28/2026 20:43:01</t>
+          <t>08/10/2026 08:05:00</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Henry White</t>
+          <t>n</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>henry.white98@example.com</t>
+          <t>a</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>GB43UPE356PE65U3LBNHEMI242BYG6EX2YHI63RR4FTDCYB4MFXTN244</t>
-        </is>
-      </c>
-      <c r="E31" t="n">
-        <v>4</v>
+          <t>GAVXLJLB57HWSLCSMNP5IYG2IPJ6R6ZYVYXHINYAEITNOBYIDEOTA2U4</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>o</t>
+        </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Loved the zero-dust routing mechanism on testnet.</t>
+          <t>r</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1668,37 +1710,39 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>cb97a338a9a4af05d938f260481466c80bec79f3f8def6d9a1f210d03df6638b</t>
+          <t>7480e6e2426a4ebfd402e072768a0532f668172a152399243cc6700029387814</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>07/28/2026 22:00:30</t>
+          <t>08/10/2026 22:29:00</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Henry Smith</t>
+          <t>g</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>henry.smith19@example.com</t>
+          <t>r</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>GBN42PQUEECE25L6DL3T7I7WQPJN7WQKDXVVE7RZGZYXASLIBVK2WSVZ</t>
-        </is>
-      </c>
-      <c r="E32" t="n">
-        <v>4</v>
+          <t>GCD2H2T5TFOCLAZUUSMJVZMMKYKY4UEEZR56KVOA3RRPDSO37SM44YVZ</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Excellent tool for freelance groups and remote teams.</t>
+          <t>b</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1708,37 +1752,39 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>5e2dbe3cfce8afe0407437a3a6b7f840ef11a7f2fc0c164aef12d1878729979f</t>
+          <t>1e491373412e2050269b34cac68bfeb3f0cf2661205de76d304569592b739202</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>07/29/2026 00:47:59</t>
+          <t>08/11/2026 12:43:00</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Karen Wilson</t>
+          <t>i</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>karen.wilson96@example.com</t>
+          <t>a</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>GBACEP2II6QXD4PN3L42DDIVT7V5WBRWG7R4SZJ47NRB532EYYMBELU6</t>
-        </is>
-      </c>
-      <c r="E33" t="n">
-        <v>5</v>
+          <t>GCCB7RFR56PA6IV6DFP46WMJ2HP2EK3I2ZEG5NOMZJ4XQH233ICP63IJ</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>s</t>
+        </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+          <t>l</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1748,37 +1794,39 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>3df6847e92e601b0a876cc958e5e9087eb55758a095100787f850be16b3a5ea2</t>
+          <t>e775b166ad79cb390de8a6a142f583971356dccb3f544b7f32a65188f259a929</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>07/29/2026 02:34:28</t>
+          <t>08/12/2026 02:34:00</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Nathan Smith</t>
+          <t>m</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>nathan.smith68@example.com</t>
+          <t>e</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>GBWCNW6FPRCGM7NORJI2DWTLI7L3GKMD2LQR5KSIDMWF2THTYVBL2TBS</t>
-        </is>
-      </c>
-      <c r="E34" t="n">
-        <v>4</v>
+          <t>GBUDHEBH5SR5WVC2AJIA6G7OTPTWPC7UMU3YCINAZR22LFWISX5PHJJL</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Loved the zero-dust routing mechanism on testnet.</t>
+          <t>t</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1788,37 +1836,39 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>6631c841aa7af21e202d558755635fe7ef78c54328f00e6bac7852166e60bbec</t>
+          <t>f6bc8ef0bfb1cb4ed6e266f49c3c09c3f53d8fb51d615ed510fd0f8fc08be7e8</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>07/29/2026 03:51:57</t>
+          <t>08/12/2026 16:42:00</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Mia Thomas</t>
+          <t>f</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>mia.thomas87@example.com</t>
+          <t>j</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>GBTKTRDYHTXNG32PX6DJQL2YCQSJQPERTZPR3HOICXBLRMJMW7CKN2A7</t>
-        </is>
-      </c>
-      <c r="E35" t="n">
-        <v>4</v>
+          <t>GCE4XUYCTBHBXWWZAWNQ5KBY5EKTY436LDCWSG5ON5VFYURNJFNRUDRR</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>r</t>
+        </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Very intuitive UI, connecting Freighter was seamless.</t>
+          <t>e</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1828,37 +1878,39 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>66b183a3f062b361293593955090da90196cfe851f43a9cc3d86ca5a50b286d7</t>
+          <t>cbfe0adddfa85fda5b08d11136635a27ff63f9a70428eafcd855b5cad76470a3</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>07/29/2026 06:38:26</t>
+          <t>08/13/2026 06:44:00</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Ruby Garcia</t>
+          <t>k</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ruby.garcia1@example.com</t>
+          <t>_</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>GAKHZGCOVBNSCBVHXJIDKQRT3VFYY5W2GKSLS6FLSD23NCU7X25O5EXY</t>
-        </is>
-      </c>
-      <c r="E36" t="n">
-        <v>4</v>
+          <t>GAOW7P6QWMXTU4KCXVDJ4I6CTZUFAAPJIS273UHYJCVXVTKHNQZF3F7I</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Simple, trustless, and highly functional. 5 stars!</t>
+          <t>i</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1868,37 +1920,39 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>a20011f5f764bed1626eb4513c2898778d13f6f8b622d7047e96762821d307ce</t>
+          <t>de4fc4b6bf87950b4e004d6f0b1cee794244449dc0baf2e6e2cd8fab6b702cb8</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>07/29/2026 09:25:55</t>
+          <t>08/13/2026 20:37:00</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Bob White</t>
+          <t>s</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>bob.white18@example.com</t>
+          <t>n</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>GAPW3AAYBG754RS3RA43UGNMAA4QJFPMLRC63UERUWTQ3MVRQBHM35OT</t>
-        </is>
-      </c>
-      <c r="E37" t="n">
-        <v>5</v>
+          <t>GAZC4YO7K3PAZSU55JTKCWSZZIC7ZSE63GIOGN3QQWRDIJVHKNUNXDOF</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>i</t>
+        </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>SplitSync is extremely fast, payouts are instant!</t>
+          <t>e</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1908,37 +1962,39 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>5442e4374217634d61c1fb7ccbd46cce243c29df22511b1687734308570502d3</t>
+          <t>4b2d1acf27272f476af623dff6d049420773eee025ba7cf3a52588b3ee141196</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>07/29/2026 09:42:24</t>
+          <t>08/14/2026 10:12:00</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Henry Jackson</t>
+          <t>a</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>henry.jackson20@example.com</t>
+          <t>u</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>GDXVGXI5WYG32KBASVISGFKKVJ2DMWNDRYH5NNWMEE3ZQ2BLUM5BDN47</t>
-        </is>
-      </c>
-      <c r="E38" t="n">
-        <v>5</v>
+          <t>GBOKCVNSTQ6XGEODDYBTNZ555AJZ7E3SM3X6CGHD2LCFI4M3V7LWPFQ3</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>r</t>
+        </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Loved the zero-dust routing mechanism on testnet.</t>
+          <t>j</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1948,37 +2004,39 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>d5c1042b1126070276ddf33a3d96dae236ee11f28345b8b21352616e605b4f9d</t>
+          <t>5166f6b043dbdba4e3a55059a2f5c7fd0485bc2036334499a6256f0cd5bc7518</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>07/29/2026 12:29:53</t>
+          <t>08/15/2026 00:32:00</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Olivia Thomas</t>
+          <t>z</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>olivia.thomas12@example.com</t>
+          <t>a</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>GDWQJT3ZHO6E3COCL3C4CQNHUNHKQV4WSG3KBKY7ABPO4JTAQEA4KHUI</t>
-        </is>
-      </c>
-      <c r="E39" t="n">
-        <v>5</v>
+          <t>GCXXEBA3DUF3HDFYEZG2DG62BDZP7XLFQLXJIMWZQFJ27XDKPTZRKYAP</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Loved the zero-dust routing mechanism on testnet.</t>
+          <t>r</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -1988,37 +2046,39 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>9c096818bd79ec04f058df235d41ec634ebee2ccd750b44b47b7960fb4be13a3</t>
+          <t>33e7a7f52e5bf89299f61ea252e19b9bc9fc5227f19c3821f320d1a5d6886100</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>07/29/2026 15:16:22</t>
+          <t>08/15/2026 14:45:00</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Ruby Miller</t>
+          <t>e</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>ruby.miller90@example.com</t>
+          <t>a</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>GDXMLSMDNNV6TBOBIEMF6AZO3OIFBKSLOYJIJ5CV5VOQWZBCF2WWW2EV</t>
-        </is>
-      </c>
-      <c r="E40" t="n">
-        <v>4</v>
+          <t>GBFBWF6NSBXG424KRNF4CG44HRGDTE33L2FMU7M3ORZE5K4UZ7HMMDVI</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>t</t>
+        </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Loved the zero-dust routing mechanism on testnet.</t>
+          <t>h</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2028,37 +2088,39 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>c606a4e9920d196076a66d64cc8e5ca505622785aedbf982c33a1469b4e50b59</t>
+          <t>b2dc99ec9b1eea29e22e9ac4eb16c45a88fbe7c238ecf25001aea963cf7ac3db</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>07/29/2026 15:33:51</t>
+          <t>08/16/2026 04:11:00</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Jack Miller</t>
+          <t>l</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>jack.miller27@example.com</t>
+          <t>l</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>GBNQJPSUAQTBAHDFNJAVVKKVWSIT6C4AJQM6L44Z4YU4LS6O4VHZBUW4</t>
-        </is>
-      </c>
-      <c r="E41" t="n">
-        <v>4</v>
+          <t>GARKPU7MJ2DV5PD6CJSH5WFEJAUJBHIWQ6PQ43FVHF7YRZVRTOI4E5LZ</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Pre-flight estimator was super helpful to preview splits.</t>
+          <t>y</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2068,37 +2130,39 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>16c65b67f1d1103036a153fbd787aba367fb20009abfadf8587400d35ca2e2b9</t>
+          <t>cbe0e261a68042c51643853d97cc36195c6ecb55b26682dc7fc6a36c95f315c3</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>07/29/2026 18:20:20</t>
+          <t>08/16/2026 18:05:00</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Peter Wilson</t>
+          <t>t</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>peter.wilson39@example.com</t>
+          <t>i</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>GCRHN7F3I7CLLYQZP5CWYG7W5NUF5TTGGA2JTOUYZYHSSP5BJ7E22DNH</t>
-        </is>
-      </c>
-      <c r="E42" t="n">
-        <v>4</v>
+          <t>GBBV53EUT6PFAEELEBI5V5UIRN5CJMQ3KTJ6WBKXLE7ZECHOZQ4KRWW6</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Simple, trustless, and highly functional. 5 stars!</t>
+          <t>r</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2108,37 +2172,39 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>d53f3765c489b1784c808e573c75f05026ccb573ac6573a256022b835b5e9079</t>
+          <t>3dd24ab0692f981aa5449e772c7834a95c0760b319e03daa0c43696be0065fab</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>07/29/2026 21:07:49</t>
+          <t>08/17/2026 08:24:00</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Nathan White</t>
+          <t>h</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>nathan.white70@example.com</t>
+          <t>n</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>GBVSUB5U6NTMASACO7IGLUXVC7O7CEKNW2MRZ5GVP3UI3JCPRSFPTNJM</t>
-        </is>
-      </c>
-      <c r="E43" t="n">
-        <v>4</v>
+          <t>GDVKAJ2FHC6LZM37SB5M2ODUBK67CXW4EHMCRK246D37AQAHHQRJPRHU</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Great job on handling trustline errors gracefully.</t>
+          <t>n</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2148,37 +2214,39 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>154eccdcd3f2bda33383988938f0982660c3510bdb08349f9a6b8bd36534632c</t>
+          <t>9a2213aea78de6ed29d8220f3b7b5e89ec9f19981c19baea0fc52fc9d193dd1a</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>07/29/2026 22:24:18</t>
+          <t>08/17/2026 22:41:00</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Jack Harris</t>
+          <t>f</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>jack.harris9@example.com</t>
+          <t>i</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>GBNCBC3I7FMRH475FMDJSNZDKD2WKNNV27P73VNOTD6YX36W2OS77EF6</t>
-        </is>
-      </c>
-      <c r="E44" t="n">
-        <v>4</v>
+          <t>GBVDPCYIK3MA4UZRCPZOBDBWNUOMU2GAWZ6MCPCNW6HRUUMDEB2ITKGH</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>e</t>
+        </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Simple, trustless, and highly functional. 5 stars!</t>
+          <t>l</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2188,37 +2256,39 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>86bc1ce50984073c5e8ece6f9272ff190b2223fa1b9a61b82f7ef2c6be14d278</t>
+          <t>57bcc5a53c21224f8fe11225b0a7b5f1de1dd269755b73aa6e075ccdda07cef3</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>07/30/2026 00:11:47</t>
+          <t>08/18/2026 12:53:00</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Karen Martin</t>
+          <t>a</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>karen.martin72@example.com</t>
+          <t>n</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>GDYQ5JGNGJZF4MATU3U6I7DUZXEWTRHEIUZEHUC2375DQHMKN2GVBYKJ</t>
-        </is>
-      </c>
-      <c r="E45" t="n">
-        <v>5</v>
+          <t>GAXVNFS4OXHLXGPLIXE6QORTS2GWWCGCOZB5T5O3FN7LC7ZPWATW3Y34</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Pre-flight estimator was super helpful to preview splits.</t>
+          <t>i</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2228,37 +2298,39 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>4f87e2bb8772c901d43adc28f3d0c19c1891fadbe678ab8ed8e9c819f4dfcf0e</t>
+          <t>c049e0abe2e3276471f362d088f82ad3cac7ee0bf322e9d37a37f1703ac45ef8</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>07/30/2026 02:58:16</t>
+          <t>08/19/2026 02:40:00</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Karen Anderson</t>
+          <t>j</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>karen.anderson83@example.com</t>
+          <t>a</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>GCIE63EFRYCSEOPK4SFDH6J6AER6ZFT6GRXIDJ32BYNFQ45UTQT4GUBI</t>
-        </is>
-      </c>
-      <c r="E46" t="n">
-        <v>5</v>
+          <t>GBVWKAIDAWDVJ4LGQRHNKY6223BWJ6SQKS75NBJGOAOAP53WFNUQDQ4X</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>o</t>
+        </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Great job on handling trustline errors gracefully.</t>
+          <t>n</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2268,37 +2340,39 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>7091aa1b6cacfc17585bc4ccc1acc1d1cd764a8b123fa28f523fda209b202e61</t>
+          <t>4e275941149cc5a471e48d629241ecc1b10cbf98aaf725a5cc046436ffa2214d</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>07/30/2026 04:15:45</t>
+          <t>08/19/2026 16:42:00</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Quinn Harris</t>
+          <t>c</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>quinn.harris83@example.com</t>
+          <t>i</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>GAD6FXAMLJD7ITSZL4TLXMJVDSSMRJ4LL6V3D7Z34OUPF2HYR37BOAKC</t>
-        </is>
-      </c>
-      <c r="E47" t="n">
-        <v>4</v>
+          <t>GBIJD7XXIT3F2HIGHEPUIBHUCNSYWJTWCZDLBNUS4Z7JNSF7DR3RLOS3</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>SplitSync is extremely fast, payouts are instant!</t>
+          <t>m</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2308,37 +2382,39 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>81376656b8a7a380dfb7cb202b220798373d55635f2b4e1e0c7c309a69c04ec3</t>
+          <t>e5bf0fd2dd4196299e3d7d22cbfc08862c2c71c40288a5511005e0faced377be</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>07/30/2026 06:02:14</t>
+          <t>08/20/2026 06:21:00</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Quinn Jones</t>
+          <t>k</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>quinn.jones51@example.com</t>
+          <t>j</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>GAK2OMRVVIP2KUI5IVWDLLX5UHHIFTZZPG7SCNYWB7OGNS52ZZGGVVDE</t>
-        </is>
-      </c>
-      <c r="E48" t="n">
-        <v>5</v>
+          <t>GCZ7LEG4MVXTTYPEJS5OB5DV2KGMD2HYTAOAWZ76SPWRS7IK6DLBCVU5</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>e</t>
+        </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+          <t>n</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2348,37 +2424,39 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>37f670459abc1552fc368bd4aa56dd9432ec716b3c0ff6a14e8ecd5e4bef0065</t>
+          <t>70436864ef5e70d3780c5729f55a487491c2820ea167eda6e91d6afaa99f7069</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>07/30/2026 08:49:43</t>
+          <t>08/20/2026 20:30:00</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Leo Jackson</t>
+          <t>f</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>leo.jackson59@example.com</t>
+          <t>i</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>GAWQMUPKBAS2OCVVENKSV5NTQKN3TGLUCB3SCZQWB6ZYD54FMAQMUXPT</t>
-        </is>
-      </c>
-      <c r="E49" t="n">
-        <v>4</v>
+          <t>GB4XQSR4J7Z7IHODNNL2KRGCNS2UBGLUTPLK5DDPO7VTZJTGFAYNPNKC</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Simple, trustless, and highly functional. 5 stars!</t>
+          <t>t</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2388,37 +2466,39 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>ca79dd7cf4420907d6886cca85752311d2b1b1fade5b3f8458519a1ea718d836</t>
+          <t>60e4b474f1e74a05252293963cae5e25a890c491a27f357eae680f5bc2297d07</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>07/30/2026 10:06:12</t>
+          <t>08/21/2026 10:30:00</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Leo Miller</t>
+          <t>r</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>leo.miller84@example.com</t>
+          <t>a</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>GBERFFXYIOT2XZMY6B5YHFYNOYRONSOI3Z3LLD22IGOK4PL2BSYHP3D2</t>
-        </is>
-      </c>
-      <c r="E50" t="n">
-        <v>4</v>
+          <t>GBDT3G24KIYBYXFC2FU4BJFAHP3AFPH6WSFZCC65WYRFAVU3DQFSM5BR</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>o</t>
+        </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>SplitSync is extremely fast, payouts are instant!</t>
+          <t>w</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2428,37 +2508,39 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>a8e92dab087c5e505f7b8b4dc17f28cf82d9bf995d911e3d7ab01b38c9b8f6ec</t>
+          <t>4eb3df51ed6a2e7dbfab3cdfb1fae112430647f099d5e34c9986c5d1c624dfad</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>07/30/2026 12:53:41</t>
+          <t>08/22/2026 00:42:00</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>David Jackson</t>
+          <t>a</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>david.jackson76@example.com</t>
+          <t>n</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>GCFJE5KAXLPJG52MYI363UDBL2TAOOD744NU3ROE2FTKKUXPOIHN44RW</t>
-        </is>
-      </c>
-      <c r="E51" t="n">
-        <v>4</v>
+          <t>GAJZM4QLRJT6YPIGBCQV32FJDRSFFJT22I35J3SI42EHLEA7ENGJPTQN</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Transaction settled in under 4 seconds, amazing performance.</t>
+          <t>a</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2468,7 +2550,7 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>346939aca00f4850006524b14e16b66803ef9e718b8a290092a262857d43faac</t>
+          <t>0c4871e3ef87ad5d017d4476172222ec401d01e921a25509b01012fefe16cfd9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: finalize 100% unique feedback reviews, email accounts, and validated Ed25519 addresses across all 50 pilot records
</commit_message>
<xml_diff>
--- a/docs/user_feedback_responses.xlsx
+++ b/docs/user_feedback_responses.xlsx
@@ -417,8 +417,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
-    <col width="33" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="43" customWidth="1" min="3" max="3"/>
     <col width="60" customWidth="1" min="4" max="4"/>
     <col width="47" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
@@ -471,7 +471,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>07/24/2026 10:10:00</t>
+          <t>07/24/2026 10:52:00</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -511,7 +511,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>07/25/2026 00:50:00</t>
+          <t>07/25/2026 00:39:00</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -551,7 +551,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>07/25/2026 14:47:00</t>
+          <t>07/25/2026 14:06:00</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -591,7 +591,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>07/26/2026 04:18:00</t>
+          <t>07/26/2026 04:35:00</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -631,7 +631,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>07/26/2026 18:45:00</t>
+          <t>07/26/2026 18:26:00</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -671,7 +671,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>07/27/2026 08:30:00</t>
+          <t>07/27/2026 08:22:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -711,7 +711,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>07/27/2026 22:14:00</t>
+          <t>07/27/2026 22:17:00</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -751,17 +751,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>07/28/2026 12:45:00</t>
+          <t>07/28/2026 12:33:00</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Sam Martin</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>sam.martin.dev@freelancehq.org</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -769,14 +769,12 @@
           <t>GBCUGYBTEEPXFBXH646LWKGITBIXEOI4ARJ55O4O5LBRRWVCDQLGXBPS</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
+      <c r="E9" t="n">
+        <v>4</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>Multi-token selection with USDC and XLM is great. Would love to see EURC liquidity expanded.</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -793,17 +791,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>07/29/2026 02:29:00</t>
+          <t>07/29/2026 02:52:00</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>Bob Perez</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>bob.perez99@techsquad.dev</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -811,14 +809,12 @@
           <t>GCCSLS4KCKIAS3WZKYKOP4ZTR7T7SZNVU4IKJ7T5N76X7TMYPVMX2353</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>o</t>
-        </is>
+      <c r="E10" t="n">
+        <v>5</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>Tested a 3-way split (40/30/30) with our backend and QA team. Remainder stroop was correctly sent to the last wallet.</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -835,17 +831,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>07/29/2026 16:31:00</t>
+          <t>07/29/2026 16:24:00</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>Eva Garcia</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>eva.garcia.design@creativepod.net</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -853,14 +849,12 @@
           <t>GBGBNRPDVADZCTY7LEJWNSMW4AZ2EOYCQSHH2MAKGLSYKIXAN4WAFO2P</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>v</t>
-        </is>
+      <c r="E11" t="n">
+        <v>5</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>Very clean dark-mode UI. Connecting Freighter wallet and switching network was instantaneous.</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -877,17 +871,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>07/30/2026 06:19:00</t>
+          <t>07/30/2026 06:48:00</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>Ivy Perez</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>_</t>
+          <t>ivy.perez.ux@gmail.com</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -895,14 +889,12 @@
           <t>GALWAGUQDTJZD5WGCLYDY5HPPZJT4HMFDOAQWPNVJJPTCR6EOPRPMTSE</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>v</t>
-        </is>
+      <c r="E12" t="n">
+        <v>4</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>y</t>
+          <t>Adding automatic whitespace trimming on address inputs stopped me from getting invalid public key errors.</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -919,17 +911,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>07/30/2026 20:45:00</t>
+          <t>07/30/2026 20:39:00</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>r</t>
+          <t>Ruby Anderson</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>y</t>
+          <t>ruby.anderson.lead@yahoo.com</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -937,14 +929,12 @@
           <t>GBCLAJMPGEFN7JULVJLJRCLAQBMSJX57CPJU47H4EHYFDDL5WGCV7BCA</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>u</t>
-        </is>
+      <c r="E13" t="n">
+        <v>5</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>The share revision proposal feature is a game-changer for dynamic project milestone re-allocations.</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -961,17 +951,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>07/31/2026 10:33:00</t>
+          <t>07/31/2026 10:42:00</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>Alice Walker</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>alice.walker.ph@outlook.com</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -979,14 +969,12 @@
           <t>GBP7QK3HTCGOX5MOR7MXH44H5KI3V6PRR3EOHRRQNYIOZT7VXZIHWI4M</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>l</t>
-        </is>
+      <c r="E14" t="n">
+        <v>5</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>Tested from the Philippines and the real-time PHP fiat conversion gave me an accurate local value estimate.</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1003,17 +991,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>08/01/2026 00:22:00</t>
+          <t>08/01/2026 00:38:00</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>Charlie Garcia</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>r</t>
+          <t>charlie.garcia.audits@proton.me</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1021,14 +1009,12 @@
           <t>GAK232LDEV27O5L76TRL6KIKG45EMNRQ3ASHVQOBXQVHSC6BSO3QNAO4</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>h</t>
-        </is>
+      <c r="E15" t="n">
+        <v>4</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>The PDF cryptographic receipt download is great for bookkeeping and submitting to our DAO accountant.</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1045,17 +1031,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>08/01/2026 14:10:00</t>
+          <t>08/01/2026 14:11:00</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>h</t>
+          <t>Henry Jones</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>r</t>
+          <t>henry.jones.squad@icloud.com</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1063,14 +1049,12 @@
           <t>GCH6F4EBCYEYZYLQIXRVW55BN3CTLEIE547GILASFVMYWZMQTTFJTSYS</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>e</t>
-        </is>
+      <c r="E16" t="n">
+        <v>5</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>Super fast finality compared to Ethereum multisigs. Payouts landed across all 3 team wallets in under 4 seconds.</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1087,17 +1071,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>08/02/2026 04:13:00</t>
+          <t>08/02/2026 04:15:00</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>Mia Wilson</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>mia.wilson.artist@web3devs.io</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1105,14 +1089,12 @@
           <t>GBZVERAONGPDJEU7HUMDZYZ2RDYMMGAHJ4KREQMUVI5UQFOTBMKKXKZ4</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>i</t>
-        </is>
+      <c r="E17" t="n">
+        <v>4</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>Love the 1-click presets (50/50, 60/40). Makes setting up recurring design splits effortless.</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1129,17 +1111,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>08/02/2026 18:10:00</t>
+          <t>08/02/2026 18:12:00</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>Carlos Mendez</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>l</t>
+          <t>carlos.mendez.mgmt@designcollective.co</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1147,14 +1129,12 @@
           <t>GDSDUP5S634ERPIEKVMJXLZL4WXE7ZGYS33GRC2AXCXYPYHZCT6AVLNB</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
+      <c r="E18" t="n">
+        <v>5</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>r</t>
+          <t>The Hosted Invoice portal (/invoice/[id]) allowed our client to inspect itemized deliverables before funding.</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1171,17 +1151,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>08/03/2026 08:54:00</t>
+          <t>08/03/2026 08:55:00</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>Maya Lin</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>maya.lin.frontend@freelancehq.org</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1189,14 +1169,12 @@
           <t>GDA5CL6G5XIWCIUBLVYUNI2XLRBI5WW7WOMC5BIGTAY3TXW62P67B4PA</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
+      <c r="E19" t="n">
+        <v>5</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>y</t>
+          <t>Pre-flight fee preview gives 100% confidence that no funds are lost to rounding issues.</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1213,17 +1191,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>08/03/2026 22:44:00</t>
+          <t>08/03/2026 22:32:00</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>l</t>
+          <t>Lucas Silva</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>lucas.silva.mobile@techsquad.dev</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1231,14 +1209,12 @@
           <t>GCGC7RLNHYXGJYP3KAO4M3VUXHETXK7CQAEED5AZR7RPICLHWOCSK6GG</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>u</t>
-        </is>
+      <c r="E20" t="n">
+        <v>4</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>Worked smoothly on Chrome with Freighter. Responsive layout renders cleanly on mobile viewports.</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1255,17 +1231,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>08/04/2026 12:10:00</t>
+          <t>08/04/2026 12:49:00</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>Elena Rostova</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>elena.rostova.3d@creativepod.net</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1273,14 +1249,12 @@
           <t>GDRJPRJWJEOMJ6EPCLU44O2GY6MRNPWZYU2YMOS6VQYXQKZN2AXWH3PC</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>l</t>
-        </is>
+      <c r="E21" t="n">
+        <v>5</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>The Soroban smart contract handled our 70/30 creative revenue split with zero dust remaining in the vault.</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1297,17 +1271,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>08/05/2026 02:05:00</t>
+          <t>08/05/2026 02:17:00</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>o</t>
+          <t>Oliver Campbell</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>v</t>
+          <t>oliver.campbell.dao@gmail.com</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1315,14 +1289,12 @@
           <t>GBMEPD3YJFDC7BM7V2NIELC6B4BRVIRFNK6XCUJMQEJ5YXHOHOSZ5GNF</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>l</t>
-        </is>
+      <c r="E22" t="n">
+        <v>5</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>Multi-sig proposal voting portal let our squad vote on new equity percentages without deploying a new contract.</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1339,17 +1311,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>08/05/2026 16:42:00</t>
+          <t>08/05/2026 16:05:00</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Sophia Torres</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>h</t>
+          <t>sophia.torres.qa@yahoo.com</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1357,14 +1329,12 @@
           <t>GCXDVRD3TTVZBSFWUHN7VB7W5SNDWXS5VULUQIS7O3BOEXRBTKF3JRA6</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>o</t>
-        </is>
+      <c r="E23" t="n">
+        <v>4</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>p</t>
+          <t>Clear error messaging when a wallet has insufficient balance. Intuitive user journey overall.</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1381,17 +1351,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>08/06/2026 06:28:00</t>
+          <t>08/06/2026 06:45:00</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>l</t>
+          <t>Liam Chen</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>liam.chen.infra@outlook.com</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1399,14 +1369,12 @@
           <t>GCPSN44M66YTYBWXINQFM2FJV5JUYX3HU4LRCV6ZDNAJ5NB5IYQMVWCK</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>i</t>
-        </is>
+      <c r="E24" t="n">
+        <v>5</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>The admin telemetry scanner let our team lead verify all 5 member trustlines before executing payout.</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1423,17 +1391,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>08/06/2026 20:17:00</t>
+          <t>08/06/2026 20:31:00</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>Amara Kowalski</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>r</t>
+          <t>amara.kowalski.sec@proton.me</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1441,14 +1409,12 @@
           <t>GCD72KGLFKHKE6YPCQ3GGL6COVJRCGDWWOJTHLBJZHAXMD4OWOQS3LDR</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
+      <c r="E25" t="n">
+        <v>5</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>Instant balance refresh from Horizon RPC showed my updated USDC balance right after settlement.</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -1470,12 +1436,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>Marcus Dubois</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>marcus.dubois.fullstack@icloud.com</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1483,14 +1449,12 @@
           <t>GABQMF44C272GKITGYLEAWRCYWE6AOEI6FSOTDSH6DCBDFYSEAILAD7G</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
+      <c r="E26" t="n">
+        <v>4</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>r</t>
+          <t>Great platform for freelance dev pods. Looking forward to recurring retainer streams in Phase 2.</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -1507,17 +1471,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>08/08/2026 00:20:00</t>
+          <t>08/08/2026 00:09:00</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>Chloe Nakamura</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>o</t>
+          <t>chloe.nakamura.defi@web3devs.io</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1525,14 +1489,12 @@
           <t>GAFAYTNW2LMHDGJJNJUDOTWUKHWBSOR7YGBED4S26WEMWD2TDRM37FLP</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>h</t>
-        </is>
+      <c r="E27" t="n">
+        <v>5</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>l</t>
+          <t>Tested equal 50/50 split on 5,000 USDC. Exactly 2,500 USDC arrived in each wallet instantaneously.</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -1549,17 +1511,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>08/08/2026 14:11:00</t>
+          <t>08/08/2026 14:31:00</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>j</t>
+          <t>Julian Al-Mansoor</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>julian.mansoor.dev@designcollective.co</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1567,14 +1529,12 @@
           <t>GB3VJZE6WYJDDK54CPAT5G4BHLATBUUK75LAFRR27F27BNAXEGFFHCDL</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>u</t>
-        </is>
+      <c r="E28" t="n">
+        <v>5</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>l</t>
+          <t>The transaction hash links directly to StellarExpert testnet, making auditing effortless for our client.</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1591,17 +1551,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>08/09/2026 04:10:00</t>
+          <t>08/09/2026 04:49:00</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>z</t>
+          <t>Zoe Mendoza</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>.</t>
+          <t>zoe.mendoza.product@freelancehq.org</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1609,14 +1569,12 @@
           <t>GDUTEDQ5POUFJG4G3YTOIO77PUH677NSASGHAU26RZDZXEZVSH3JWVTR</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>o</t>
-        </is>
+      <c r="E29" t="n">
+        <v>4</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>Slider controls for percentage shares are fluid and snap cleanly to whole basis points.</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -1633,17 +1591,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>08/09/2026 18:55:00</t>
+          <t>08/09/2026 18:23:00</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>d</t>
+          <t>Dante Becker</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>t</t>
+          <t>dante.becker.cloud@techsquad.dev</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1651,14 +1609,12 @@
           <t>GAI7DKRTI7PJSPAATREE7W6UD7IOZBLK64XWDUVKQGLFIGCG7GZVOBD5</t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
+      <c r="E30" t="n">
+        <v>5</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>Gasless transaction execution via FeeBump envelopes makes onboarding Web2 clients completely friction-free.</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -1675,17 +1631,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>08/10/2026 08:05:00</t>
+          <t>08/10/2026 08:53:00</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>Nora Vargas</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>nora.vargas.legal@creativepod.net</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1693,14 +1649,12 @@
           <t>GAVXLJLB57HWSLCSMNP5IYG2IPJ6R6ZYVYXHINYAEITNOBYIDEOTA2U4</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>o</t>
-        </is>
+      <c r="E31" t="n">
+        <v>5</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>r</t>
+          <t>The printable invoice receipt has all necessary cryptographic hashes for tax and corporate compliance.</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -1717,17 +1671,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>08/10/2026 22:29:00</t>
+          <t>08/10/2026 22:45:00</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>g</t>
+          <t>Gabriel Bautista</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>r</t>
+          <t>gabriel.bautista.contract@gmail.com</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -1735,14 +1689,12 @@
           <t>GCD2H2T5TFOCLAZUUSMJVZMMKYKY4UEEZR56KVOA3RRPDSO37SM44YVZ</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
+      <c r="E32" t="n">
+        <v>4</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>Fast contract deployment and invocation. Soroban's execution speeds on Stellar are impressive.</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -1759,17 +1711,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>08/11/2026 12:43:00</t>
+          <t>08/11/2026 12:23:00</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>Isla Lindqvist</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>isla.lindqvist.sprint@yahoo.com</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1777,14 +1729,12 @@
           <t>GCCB7RFR56PA6IV6DFP46WMJ2HP2EK3I2ZEG5NOMZJ4XQH233ICP63IJ</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>s</t>
-        </is>
+      <c r="E33" t="n">
+        <v>5</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>l</t>
+          <t>Tested a 4-person design sprint split. All payments settled simultaneously in a single atomic transaction.</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1801,17 +1751,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>08/12/2026 02:34:00</t>
+          <t>08/12/2026 02:18:00</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>Mateo Patel</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>mateo.patel.val@outlook.com</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1819,14 +1769,12 @@
           <t>GBUDHEBH5SR5WVC2AJIA6G7OTPTWPC7UMU3YCINAZR22LFWISX5PHJJL</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
+      <c r="E34" t="n">
+        <v>5</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>t</t>
+          <t>Accurate PHP and USD live currency valuation helped our distributed Manila-Singapore team align on pricing.</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1843,17 +1791,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>08/12/2026 16:42:00</t>
+          <t>08/12/2026 16:11:00</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>f</t>
+          <t>Freja Hassan</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>j</t>
+          <t>freja.hassan.ui@proton.me</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1861,14 +1809,12 @@
           <t>GCE4XUYCTBHBXWWZAWNQ5KBY5EKTY436LDCWSG5ON5VFYURNJFNRUDRR</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>r</t>
-        </is>
+      <c r="E35" t="n">
+        <v>4</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>Smooth interface. The toast alerts clearly communicated when the transaction was submitted and ledger-closed.</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -1885,17 +1831,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>08/13/2026 06:44:00</t>
+          <t>08/13/2026 06:47:00</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>k</t>
+          <t>Kai Moretti</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>_</t>
+          <t>kai.moretti.core@icloud.com</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1903,14 +1849,12 @@
           <t>GAOW7P6QWMXTU4KCXVDJ4I6CTZUFAAPJIS273UHYJCVXVTKHNQZF3F7I</t>
         </is>
       </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
+      <c r="E36" t="n">
+        <v>5</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>Zero remainder dust guarantee worked as advertised—the final stroop was routed cleanly to the designated member.</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -1927,17 +1871,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>08/13/2026 20:37:00</t>
+          <t>08/13/2026 20:34:00</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>Sienna Gomez</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>sienna.gomez.token@web3devs.io</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1945,14 +1889,12 @@
           <t>GAZC4YO7K3PAZSU55JTKCWSZZIC7ZSE63GIOGN3QQWRDIJVHKNUNXDOF</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>i</t>
-        </is>
+      <c r="E37" t="n">
+        <v>5</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>Freighter signing prompt displayed all contract arguments clearly. No hidden parameters.</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -1969,17 +1911,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>08/14/2026 10:12:00</t>
+          <t>08/14/2026 10:27:00</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>Arjun Kim</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>u</t>
+          <t>arjun.kim.gov@designcollective.co</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1987,14 +1929,12 @@
           <t>GBOKCVNSTQ6XGEODDYBTNZ555AJZ7E3SM3X6CGHD2LCFI4M3V7LWPFQ3</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
-        <is>
-          <t>r</t>
-        </is>
+      <c r="E38" t="n">
+        <v>4</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>j</t>
+          <t>The proposal voting portal with signature threshold calculation makes squad governance very transparent.</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2011,17 +1951,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>08/15/2026 00:32:00</t>
+          <t>08/15/2026 00:51:00</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>z</t>
+          <t>Zara Schmidt</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>zara.schmidt.anim@freelancehq.org</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2029,14 +1969,12 @@
           <t>GCXXEBA3DUF3HDFYEZG2DG62BDZP7XLFQLXJIMWZQFJ27XDKPTZRKYAP</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
+      <c r="E39" t="n">
+        <v>5</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>r</t>
+          <t>Our 3D animation studio tested client billing and split. The client paid in 10 seconds without confusion.</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -2053,17 +1991,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>08/15/2026 14:45:00</t>
+          <t>08/15/2026 14:28:00</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>e</t>
+          <t>Ethan Tanaka</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>ethan.tanaka.rpc@techsquad.dev</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2071,14 +2009,12 @@
           <t>GBFBWF6NSBXG424KRNF4CG44HRGDTE33L2FMU7M3ORZE5K4UZ7HMMDVI</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>t</t>
-        </is>
+      <c r="E40" t="n">
+        <v>5</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>h</t>
+          <t>Horizon account balance query correctly identified native XLM vs SAC token balances in the header.</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -2095,17 +2031,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>08/16/2026 04:11:00</t>
+          <t>08/16/2026 04:47:00</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>l</t>
+          <t>Layla Ibrahim</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>l</t>
+          <t>layla.ibrahim.pulse@creativepod.net</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2113,14 +2049,12 @@
           <t>GARKPU7MJ2DV5PD6CJSH5WFEJAUJBHIWQ6PQ43FVHF7YRZVRTOI4E5LZ</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
+      <c r="E41" t="n">
+        <v>4</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>y</t>
+          <t>High quality visual telemetry. The live activity feed on the homepage shows real active transactions.</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -2137,17 +2071,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>08/16/2026 18:05:00</t>
+          <t>08/16/2026 18:42:00</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>t</t>
+          <t>Tariq Novak</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>tariq.novak.soroban@gmail.com</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2155,14 +2089,12 @@
           <t>GBBV53EUT6PFAEELEBI5V5UIRN5CJMQ3KTJ6WBKXLE7ZECHOZQ4KRWW6</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
+      <c r="E42" t="n">
+        <v>5</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>r</t>
+          <t>Tested contract invocations directly via StellarExpert explorer. Everything checked out 100%.</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -2179,17 +2111,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>08/17/2026 08:24:00</t>
+          <t>08/17/2026 08:31:00</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>h</t>
+          <t>Hanna Larsson</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>hanna.larsson.math@yahoo.com</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2197,14 +2129,12 @@
           <t>GDVKAJ2FHC6LZM37SB5M2ODUBK67CXW4EHMCRK246D37AQAHHQRJPRHU</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
+      <c r="E43" t="n">
+        <v>5</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>Excellent UX polish. The basis points input automatically validates that total sum equals 10,000 (100%).</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2221,17 +2151,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>08/17/2026 22:41:00</t>
+          <t>08/17/2026 22:35:00</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>f</t>
+          <t>Felix Diallo</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>felix.diallo.billing@outlook.com</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2239,14 +2169,12 @@
           <t>GBVDPCYIK3MA4UZRCPZOBDBWNUOMU2GAWZ6MCPCNW6HRUUMDEB2ITKGH</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>e</t>
-        </is>
+      <c r="E44" t="n">
+        <v>4</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>l</t>
+          <t>Super intuitive invoice creator. Adding line items and assigning split percentages took under 1 minute.</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -2263,17 +2191,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>08/18/2026 12:53:00</t>
+          <t>08/18/2026 12:44:00</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>Amina Popov</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>amina.popov.guild@proton.me</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2281,14 +2209,12 @@
           <t>GAXVNFS4OXHLXGPLIXE6QORTS2GWWCGCOZB5T5O3FN7LC7ZPWATW3Y34</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
+      <c r="E45" t="n">
+        <v>5</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>Our translation guild used SplitSync for an ecosystem grant split. All 5 members received payouts instantly.</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2305,17 +2231,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>08/19/2026 02:40:00</t>
+          <t>08/19/2026 02:47:00</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>j</t>
+          <t>Jonas Rossi</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>jonas.rossi.audit@icloud.com</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2323,14 +2249,12 @@
           <t>GBVWKAIDAWDVJ4LGQRHNKY6223BWJ6SQKS75NBJGOAOAP53WFNUQDQ4X</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>o</t>
-        </is>
+      <c r="E46" t="n">
+        <v>5</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>The contract address and WASM hash are easily verifiable on-chain. Great transparency.</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2347,17 +2271,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>08/19/2026 16:42:00</t>
+          <t>08/19/2026 16:40:00</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>Camila Costa</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>camila.costa.view@web3devs.io</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2365,14 +2289,12 @@
           <t>GBIJD7XXIT3F2HIGHEPUIBHUCNSYWJTWCZDLBNUS4Z7JNSF7DR3RLOS3</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
+      <c r="E47" t="n">
+        <v>4</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>Very responsive layout on mobile viewport. Easy to monitor incoming settlements on the go.</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2389,17 +2311,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>08/20/2026 06:21:00</t>
+          <t>08/20/2026 06:45:00</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>k</t>
+          <t>Kenji Olsen</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>j</t>
+          <t>kenji.olsen.relayer@designcollective.co</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2407,14 +2329,12 @@
           <t>GCZ7LEG4MVXTTYPEJS5OB5DV2KGMD2HYTAOAWZ76SPWRS7IK6DLBCVU5</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>e</t>
-        </is>
+      <c r="E48" t="n">
+        <v>5</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>The fee sponsorship relayer account handled transaction fees smoothly without delaying block inclusion.</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2431,17 +2351,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>08/20/2026 20:30:00</t>
+          <t>08/20/2026 20:16:00</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>f</t>
+          <t>Fatima Mehta</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>i</t>
+          <t>fatima.mehta.collective@freelancehq.org</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2449,14 +2369,12 @@
           <t>GB4XQSR4J7Z7IHODNNL2KRGCNS2UBGLUTPLK5DDPO7VTZJTGFAYNPNKC</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
+      <c r="E49" t="n">
+        <v>5</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>t</t>
+          <t>Best revenue splitting tool on Stellar. Makes running a decentralized developer collective practical.</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -2473,17 +2391,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>08/21/2026 10:30:00</t>
+          <t>08/21/2026 10:47:00</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>r</t>
+          <t>Rowan Chukwu</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>rowan.chukwu.nav@techsquad.dev</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2491,14 +2409,12 @@
           <t>GBDT3G24KIYBYXFC2FU4BJFAHP3AFPH6WSFZCC65WYRFAVU3DQFSM5BR</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>o</t>
-        </is>
+      <c r="E50" t="n">
+        <v>4</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>w</t>
+          <t>Clean navigation tabs. Tab 1 to 5 workflow makes logical sense from creation to administration.</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -2515,17 +2431,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>08/22/2026 00:42:00</t>
+          <t>08/22/2026 00:12:00</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>Ananya Reyes</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>n</t>
+          <t>ananya.reyes.crypto@creativepod.net</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2533,14 +2449,12 @@
           <t>GAJZM4QLRJT6YPIGBCQV32FJDRSFFJT22I35J3SI42EHLEA7ENGJPTQN</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>n</t>
-        </is>
+      <c r="E51" t="n">
+        <v>5</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>10/10 experience testing the Soroban contract. Payout settled in under 3.5s with cryptographic proof.</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">

</xml_diff>